<commit_message>
feat: se cambia código formato remisiones de PA-FR-09 a PA-FR-52
</commit_message>
<xml_diff>
--- a/apps/templates/EXCEL/remisiones.xlsx
+++ b/apps/templates/EXCEL/remisiones.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SINTRA\apps\templates\EXCEL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{419B783E-BF94-4C3E-9F71-41A27B23F3B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55CDF934-C38B-4F86-9345-143E6536EA92}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3BFB0A6B-61D2-4748-9625-7D939A6F5CCD}"/>
   </bookViews>
@@ -19,17 +19,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -103,9 +92,6 @@
     <t>Fecha:                                                      6/10/2022</t>
   </si>
   <si>
-    <t>Código:                                           PA-FR-09</t>
-  </si>
-  <si>
     <t>Versión:                           3</t>
   </si>
   <si>
@@ -162,13 +148,16 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>Código:                                           PA-FR-52</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -426,77 +415,77 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -833,182 +822,182 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACF9F5A1-4611-4F3F-A852-7E08544F7F8D}">
   <dimension ref="A1:G56"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="20.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="20.69921875" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="20.6640625" style="2"/>
-    <col min="2" max="3" width="25.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" style="2"/>
-    <col min="5" max="5" width="23.44140625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="16.77734375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="26.109375" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="20.6640625" style="2"/>
+    <col min="1" max="1" width="20.69921875" style="2"/>
+    <col min="2" max="3" width="25.69921875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="20.69921875" style="2"/>
+    <col min="5" max="5" width="23.3984375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="16.796875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="26.09765625" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="20.69921875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="70.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="23"/>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="25"/>
+    <row r="1" spans="1:7" ht="70.5" customHeight="1">
+      <c r="A1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="18"/>
       <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="39.75" customHeight="1">
+      <c r="A2" s="19"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="26"/>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" s="8" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
+      <c r="B5" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="29"/>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="s">
+      <c r="B6" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="29"/>
-      <c r="D6" s="29"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="s">
+      <c r="B7" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="29"/>
-      <c r="D7" s="29"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G7" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" s="8" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="32.25" customHeight="1">
       <c r="A9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="C9" s="24"/>
+      <c r="D9" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="30"/>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G9" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" s="3"/>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
       <c r="G10" s="4"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7">
       <c r="A11" s="3"/>
-      <c r="B11" s="19"/>
-      <c r="C11" s="20"/>
+      <c r="B11" s="25"/>
+      <c r="C11" s="26"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7">
       <c r="A12" s="3"/>
-      <c r="B12" s="21"/>
-      <c r="C12" s="22"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="28"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="4"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7">
       <c r="A13" s="3"/>
-      <c r="B13" s="21"/>
-      <c r="C13" s="22"/>
+      <c r="B13" s="27"/>
+      <c r="C13" s="28"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="4"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7">
       <c r="A14" s="5"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="20"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="26"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
@@ -1017,10 +1006,10 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7">
       <c r="A15" s="5"/>
-      <c r="B15" s="19"/>
-      <c r="C15" s="20"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="26"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
@@ -1029,10 +1018,10 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7">
       <c r="A16" s="5"/>
-      <c r="B16" s="19"/>
-      <c r="C16" s="20"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="26"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
@@ -1041,7 +1030,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7">
       <c r="A17" s="5"/>
       <c r="B17" s="11"/>
       <c r="C17" s="12"/>
@@ -1053,7 +1042,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7">
       <c r="A18" s="5"/>
       <c r="B18" s="11"/>
       <c r="C18" s="12"/>
@@ -1065,7 +1054,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7">
       <c r="A19" s="5"/>
       <c r="B19" s="11"/>
       <c r="C19" s="12"/>
@@ -1077,7 +1066,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7">
       <c r="A20" s="5"/>
       <c r="B20" s="11"/>
       <c r="C20" s="12"/>
@@ -1089,7 +1078,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7">
       <c r="A21" s="5"/>
       <c r="B21" s="11"/>
       <c r="C21" s="12"/>
@@ -1101,7 +1090,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7">
       <c r="A22" s="5"/>
       <c r="B22" s="11"/>
       <c r="C22" s="12"/>
@@ -1113,10 +1102,10 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7">
       <c r="A23" s="5"/>
-      <c r="B23" s="19"/>
-      <c r="C23" s="20"/>
+      <c r="B23" s="25"/>
+      <c r="C23" s="26"/>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
@@ -1125,10 +1114,10 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7">
       <c r="A24" s="5"/>
-      <c r="B24" s="19"/>
-      <c r="C24" s="20"/>
+      <c r="B24" s="25"/>
+      <c r="C24" s="26"/>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
@@ -1137,10 +1126,10 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7">
       <c r="A25" s="5"/>
-      <c r="B25" s="19"/>
-      <c r="C25" s="20"/>
+      <c r="B25" s="25"/>
+      <c r="C25" s="26"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
@@ -1149,10 +1138,10 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7">
       <c r="A26" s="5"/>
-      <c r="B26" s="19"/>
-      <c r="C26" s="20"/>
+      <c r="B26" s="25"/>
+      <c r="C26" s="26"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
@@ -1161,10 +1150,10 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7">
       <c r="A27" s="5"/>
-      <c r="B27" s="19"/>
-      <c r="C27" s="20"/>
+      <c r="B27" s="25"/>
+      <c r="C27" s="26"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
@@ -1173,10 +1162,10 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7">
       <c r="A28" s="5"/>
-      <c r="B28" s="19"/>
-      <c r="C28" s="20"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
@@ -1185,10 +1174,10 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7">
       <c r="A29" s="5"/>
-      <c r="B29" s="19"/>
-      <c r="C29" s="20"/>
+      <c r="B29" s="25"/>
+      <c r="C29" s="26"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
@@ -1197,73 +1186,73 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7">
       <c r="A30" s="5"/>
-      <c r="B30" s="19"/>
-      <c r="C30" s="20"/>
+      <c r="B30" s="25"/>
+      <c r="C30" s="26"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
       <c r="G30" s="4"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7">
       <c r="A31" s="5"/>
-      <c r="B31" s="19"/>
-      <c r="C31" s="20"/>
+      <c r="B31" s="25"/>
+      <c r="C31" s="26"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
       <c r="G31" s="4"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7">
       <c r="A32" s="5"/>
-      <c r="B32" s="19"/>
-      <c r="C32" s="20"/>
+      <c r="B32" s="25"/>
+      <c r="C32" s="26"/>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
       <c r="G32" s="4"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7">
       <c r="A33" s="5"/>
-      <c r="B33" s="16"/>
-      <c r="C33" s="16"/>
+      <c r="B33" s="22"/>
+      <c r="C33" s="22"/>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
       <c r="G33" s="4"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7">
       <c r="A34" s="5"/>
-      <c r="B34" s="16"/>
-      <c r="C34" s="16"/>
+      <c r="B34" s="22"/>
+      <c r="C34" s="22"/>
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
       <c r="G34" s="4"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7">
       <c r="A35" s="5"/>
-      <c r="B35" s="16"/>
-      <c r="C35" s="16"/>
+      <c r="B35" s="22"/>
+      <c r="C35" s="22"/>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7">
       <c r="A36" s="6"/>
       <c r="B36" s="14"/>
       <c r="C36" s="14"/>
       <c r="D36" s="14"/>
       <c r="E36" s="15"/>
-      <c r="F36" s="17">
+      <c r="F36" s="38">
         <f>SUM(F10:F35)</f>
         <v>0</v>
       </c>
-      <c r="G36" s="18"/>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G36" s="39"/>
+    </row>
+    <row r="37" spans="1:7">
       <c r="A37" s="6"/>
       <c r="B37" s="7"/>
       <c r="C37" s="7"/>
@@ -1272,175 +1261,177 @@
       <c r="F37" s="6"/>
       <c r="G37" s="6"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" s="31" t="s">
-        <v>21</v>
-      </c>
-      <c r="B38" s="32"/>
-      <c r="C38" s="32"/>
-      <c r="D38" s="32"/>
-      <c r="E38" s="32"/>
-      <c r="F38" s="32"/>
-      <c r="G38" s="33"/>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A39" s="34"/>
-      <c r="B39" s="35"/>
-      <c r="C39" s="35"/>
-      <c r="D39" s="35"/>
-      <c r="E39" s="35"/>
-      <c r="F39" s="35"/>
-      <c r="G39" s="36"/>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A40" s="34"/>
-      <c r="B40" s="35"/>
-      <c r="C40" s="35"/>
-      <c r="D40" s="35"/>
-      <c r="E40" s="35"/>
-      <c r="F40" s="35"/>
-      <c r="G40" s="36"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A41" s="34"/>
-      <c r="B41" s="35"/>
-      <c r="C41" s="35"/>
-      <c r="D41" s="35"/>
-      <c r="E41" s="35"/>
-      <c r="F41" s="35"/>
-      <c r="G41" s="36"/>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A42" s="34"/>
-      <c r="B42" s="35"/>
-      <c r="C42" s="35"/>
-      <c r="D42" s="35"/>
-      <c r="E42" s="35"/>
-      <c r="F42" s="35"/>
-      <c r="G42" s="36"/>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A43" s="34"/>
-      <c r="B43" s="35"/>
-      <c r="C43" s="35"/>
-      <c r="D43" s="35"/>
-      <c r="E43" s="35"/>
-      <c r="F43" s="35"/>
-      <c r="G43" s="36"/>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A44" s="34"/>
-      <c r="B44" s="35"/>
-      <c r="C44" s="35"/>
-      <c r="D44" s="35"/>
-      <c r="E44" s="35"/>
-      <c r="F44" s="35"/>
-      <c r="G44" s="36"/>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A45" s="34"/>
-      <c r="B45" s="35"/>
-      <c r="C45" s="35"/>
-      <c r="D45" s="35"/>
-      <c r="E45" s="35"/>
-      <c r="F45" s="35"/>
-      <c r="G45" s="36"/>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A46" s="34"/>
-      <c r="B46" s="35"/>
-      <c r="C46" s="35"/>
-      <c r="D46" s="35"/>
-      <c r="E46" s="35"/>
-      <c r="F46" s="35"/>
-      <c r="G46" s="36"/>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A47" s="34"/>
-      <c r="B47" s="35"/>
-      <c r="C47" s="35"/>
-      <c r="D47" s="35"/>
-      <c r="E47" s="35"/>
-      <c r="F47" s="35"/>
-      <c r="G47" s="36"/>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A48" s="34"/>
-      <c r="B48" s="35"/>
-      <c r="C48" s="35"/>
-      <c r="D48" s="35"/>
-      <c r="E48" s="35"/>
-      <c r="F48" s="35"/>
-      <c r="G48" s="36"/>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A49" s="34"/>
-      <c r="B49" s="35"/>
-      <c r="C49" s="35"/>
-      <c r="D49" s="35"/>
-      <c r="E49" s="35"/>
-      <c r="F49" s="35"/>
-      <c r="G49" s="36"/>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A50" s="34"/>
-      <c r="B50" s="35"/>
-      <c r="C50" s="35"/>
-      <c r="D50" s="35"/>
-      <c r="E50" s="35"/>
-      <c r="F50" s="35"/>
-      <c r="G50" s="36"/>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A51" s="34"/>
-      <c r="B51" s="35"/>
-      <c r="C51" s="35"/>
-      <c r="D51" s="35"/>
-      <c r="E51" s="35"/>
-      <c r="F51" s="35"/>
-      <c r="G51" s="36"/>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A52" s="37"/>
-      <c r="B52" s="38"/>
-      <c r="C52" s="38"/>
-      <c r="D52" s="38"/>
-      <c r="E52" s="38"/>
-      <c r="F52" s="38"/>
-      <c r="G52" s="39"/>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7">
+      <c r="A38" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="B38" s="30"/>
+      <c r="C38" s="30"/>
+      <c r="D38" s="30"/>
+      <c r="E38" s="30"/>
+      <c r="F38" s="30"/>
+      <c r="G38" s="31"/>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" s="32"/>
+      <c r="B39" s="33"/>
+      <c r="C39" s="33"/>
+      <c r="D39" s="33"/>
+      <c r="E39" s="33"/>
+      <c r="F39" s="33"/>
+      <c r="G39" s="34"/>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" s="32"/>
+      <c r="B40" s="33"/>
+      <c r="C40" s="33"/>
+      <c r="D40" s="33"/>
+      <c r="E40" s="33"/>
+      <c r="F40" s="33"/>
+      <c r="G40" s="34"/>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" s="32"/>
+      <c r="B41" s="33"/>
+      <c r="C41" s="33"/>
+      <c r="D41" s="33"/>
+      <c r="E41" s="33"/>
+      <c r="F41" s="33"/>
+      <c r="G41" s="34"/>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" s="32"/>
+      <c r="B42" s="33"/>
+      <c r="C42" s="33"/>
+      <c r="D42" s="33"/>
+      <c r="E42" s="33"/>
+      <c r="F42" s="33"/>
+      <c r="G42" s="34"/>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43" s="32"/>
+      <c r="B43" s="33"/>
+      <c r="C43" s="33"/>
+      <c r="D43" s="33"/>
+      <c r="E43" s="33"/>
+      <c r="F43" s="33"/>
+      <c r="G43" s="34"/>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44" s="32"/>
+      <c r="B44" s="33"/>
+      <c r="C44" s="33"/>
+      <c r="D44" s="33"/>
+      <c r="E44" s="33"/>
+      <c r="F44" s="33"/>
+      <c r="G44" s="34"/>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45" s="32"/>
+      <c r="B45" s="33"/>
+      <c r="C45" s="33"/>
+      <c r="D45" s="33"/>
+      <c r="E45" s="33"/>
+      <c r="F45" s="33"/>
+      <c r="G45" s="34"/>
+    </row>
+    <row r="46" spans="1:7">
+      <c r="A46" s="32"/>
+      <c r="B46" s="33"/>
+      <c r="C46" s="33"/>
+      <c r="D46" s="33"/>
+      <c r="E46" s="33"/>
+      <c r="F46" s="33"/>
+      <c r="G46" s="34"/>
+    </row>
+    <row r="47" spans="1:7">
+      <c r="A47" s="32"/>
+      <c r="B47" s="33"/>
+      <c r="C47" s="33"/>
+      <c r="D47" s="33"/>
+      <c r="E47" s="33"/>
+      <c r="F47" s="33"/>
+      <c r="G47" s="34"/>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48" s="32"/>
+      <c r="B48" s="33"/>
+      <c r="C48" s="33"/>
+      <c r="D48" s="33"/>
+      <c r="E48" s="33"/>
+      <c r="F48" s="33"/>
+      <c r="G48" s="34"/>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49" s="32"/>
+      <c r="B49" s="33"/>
+      <c r="C49" s="33"/>
+      <c r="D49" s="33"/>
+      <c r="E49" s="33"/>
+      <c r="F49" s="33"/>
+      <c r="G49" s="34"/>
+    </row>
+    <row r="50" spans="1:7">
+      <c r="A50" s="32"/>
+      <c r="B50" s="33"/>
+      <c r="C50" s="33"/>
+      <c r="D50" s="33"/>
+      <c r="E50" s="33"/>
+      <c r="F50" s="33"/>
+      <c r="G50" s="34"/>
+    </row>
+    <row r="51" spans="1:7">
+      <c r="A51" s="32"/>
+      <c r="B51" s="33"/>
+      <c r="C51" s="33"/>
+      <c r="D51" s="33"/>
+      <c r="E51" s="33"/>
+      <c r="F51" s="33"/>
+      <c r="G51" s="34"/>
+    </row>
+    <row r="52" spans="1:7">
+      <c r="A52" s="35"/>
+      <c r="B52" s="36"/>
+      <c r="C52" s="36"/>
+      <c r="D52" s="36"/>
+      <c r="E52" s="36"/>
+      <c r="F52" s="36"/>
+      <c r="G52" s="37"/>
+    </row>
+    <row r="53" spans="1:7">
       <c r="B53" s="13"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7">
       <c r="A54" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D54" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B54" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D54" s="2" t="s">
+      <c r="E54" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E54" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="55" spans="1:7">
       <c r="B55" s="13"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7">
       <c r="B56" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A1:E2"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="A38:G52"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
@@ -1453,15 +1444,13 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B27:C27"/>
-    <mergeCell ref="A38:G52"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="A1:E2"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B9:C9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>